<commit_message>
2nd attempt at a state machine system
</commit_message>
<xml_diff>
--- a/Documents/Game Development/Godot/Smash Dungeon/SD_WorkLog.xlsx
+++ b/Documents/Game Development/Godot/Smash Dungeon/SD_WorkLog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E50B21B4-C8B9-4A91-BC12-E2A3F6363E3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE2EFFD8-AEE7-48B8-A8EC-E72CAD080C0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
   <sheets>
     <sheet name="Smash Dungeon" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="98">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -379,6 +379,25 @@
   </si>
   <si>
     <t>Adding weapon system to remaining enemies</t>
+  </si>
+  <si>
+    <t>Crawling enemy - component system</t>
+  </si>
+  <si>
+    <t>Gave up on crawling enemy
+- component system unwiedly and couldn't produce the desired functionality</t>
+  </si>
+  <si>
+    <t>Added procedural arena creations</t>
+  </si>
+  <si>
+    <t>Decided to return to save after prcedural arena system</t>
+  </si>
+  <si>
+    <t>Began refactoring to State Machine system</t>
+  </si>
+  <si>
+    <t>Continuing to trouble shoot fodder_enemy_sm</t>
   </si>
 </sst>
 </file>
@@ -517,8 +536,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G71" totalsRowShown="0">
-  <autoFilter ref="B6:G71" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G78" totalsRowShown="0">
+  <autoFilter ref="B6:G78" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
@@ -884,7 +903,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -910,8 +929,8 @@
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>SUM(G7:G71)</f>
-        <v>7.3513888888888888</v>
+        <f>SUM(G7:G78)</f>
+        <v>8.59236111111111</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -2072,7 +2091,7 @@
         <v>85</v>
       </c>
       <c r="G66" s="2">
-        <f>IF(D66&lt;C66, D66+1, D66) - C66</f>
+        <f t="shared" ref="G66:G71" si="8">IF(D66&lt;C66, D66+1, D66) - C66</f>
         <v>0.13819444444444451</v>
       </c>
     </row>
@@ -2088,7 +2107,7 @@
         <v>86</v>
       </c>
       <c r="G67" s="2">
-        <f>IF(D67&lt;C67, D67+1, D67) - C67</f>
+        <f t="shared" si="8"/>
         <v>4.8611111111111049E-2</v>
       </c>
     </row>
@@ -2107,7 +2126,7 @@
         <v>87</v>
       </c>
       <c r="G68" s="2">
-        <f>IF(D68&lt;C68, D68+1, D68) - C68</f>
+        <f t="shared" si="8"/>
         <v>9.027777777777779E-2</v>
       </c>
     </row>
@@ -2128,7 +2147,7 @@
         <v>89</v>
       </c>
       <c r="G69" s="2">
-        <f>IF(D69&lt;C69, D69+1, D69) - C69</f>
+        <f t="shared" si="8"/>
         <v>8.5416666666666696E-2</v>
       </c>
     </row>
@@ -2147,7 +2166,7 @@
         <v>90</v>
       </c>
       <c r="G70" s="2">
-        <f>IF(D70&lt;C70, D70+1, D70) - C70</f>
+        <f t="shared" si="8"/>
         <v>0.22777777777777763</v>
       </c>
     </row>
@@ -2166,22 +2185,149 @@
         <v>91</v>
       </c>
       <c r="G71" s="2">
-        <f>IF(D71&lt;C71, D71+1, D71) - C71</f>
+        <f t="shared" si="8"/>
         <v>0.59027777777777779</v>
       </c>
     </row>
     <row r="72" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B72" s="1"/>
       <c r="C72" s="2"/>
       <c r="D72" s="2"/>
-      <c r="G72" s="2"/>
+      <c r="E72" t="s">
+        <v>71</v>
+      </c>
+      <c r="F72" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="G72" s="2">
+        <f t="shared" ref="G72:G77" si="9">IF(D72&lt;C72, D72+1, D72) - C72</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="73" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="F73" s="8" t="s">
+      <c r="B73" s="1">
+        <v>45769</v>
+      </c>
+      <c r="C73" s="2">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="D73" s="2">
+        <v>0.93333333333333335</v>
+      </c>
+      <c r="E73" t="s">
+        <v>74</v>
+      </c>
+      <c r="F73" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="G73" s="2">
+        <f t="shared" si="9"/>
+        <v>0.28749999999999998</v>
+      </c>
+    </row>
+    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C74" s="2">
+        <v>0.97916666666666663</v>
+      </c>
+      <c r="D74" s="2">
+        <v>6.8750000000000006E-2</v>
+      </c>
+      <c r="E74" t="s">
+        <v>74</v>
+      </c>
+      <c r="F74" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="G74" s="2">
+        <f t="shared" si="9"/>
+        <v>8.9583333333333459E-2</v>
+      </c>
+    </row>
+    <row r="75" spans="2:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="B75" s="1">
+        <v>45770</v>
+      </c>
+      <c r="C75" s="2">
+        <v>0.63888888888888884</v>
+      </c>
+      <c r="D75" s="2">
+        <v>0.81944444444444442</v>
+      </c>
+      <c r="E75" t="s">
+        <v>74</v>
+      </c>
+      <c r="F75" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G75" s="2">
+        <f t="shared" si="9"/>
+        <v>0.18055555555555558</v>
+      </c>
+    </row>
+    <row r="76" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C76" s="2">
+        <v>0.9375</v>
+      </c>
+      <c r="D76" s="2">
+        <v>0.97916666666666663</v>
+      </c>
+      <c r="E76" t="s">
+        <v>74</v>
+      </c>
+      <c r="F76" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="G76" s="2">
+        <f t="shared" si="9"/>
+        <v>4.166666666666663E-2</v>
+      </c>
+    </row>
+    <row r="77" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B77" s="1">
+        <v>45772</v>
+      </c>
+      <c r="C77" s="2">
+        <v>0.85833333333333328</v>
+      </c>
+      <c r="D77" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E77" t="s">
+        <v>74</v>
+      </c>
+      <c r="F77" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G77" s="2">
+        <f t="shared" si="9"/>
+        <v>0.10000000000000009</v>
+      </c>
+    </row>
+    <row r="78" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B78" s="1">
+        <v>45773</v>
+      </c>
+      <c r="C78" s="2">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="E78" t="s">
+        <v>74</v>
+      </c>
+      <c r="F78" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="G78" s="2">
+        <f>IF(D78&lt;C78, D78+1, D78) - C78</f>
+        <v>0.54166666666666674</v>
+      </c>
+    </row>
+    <row r="81" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F81" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="F74" s="9" t="s">
+    <row r="82" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F82" s="9" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>

<commit_message>
began refactoring fodder enemy back to base enemy sm to integrate updates to attack and chase. Now attempting to add a telgraph state into base to then be extended in fodder enemy and others.
</commit_message>
<xml_diff>
--- a/Documents/Game Development/Godot/Smash Dungeon/SD_WorkLog.xlsx
+++ b/Documents/Game Development/Godot/Smash Dungeon/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE2EFFD8-AEE7-48B8-A8EC-E72CAD080C0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B43942-6166-40D9-ACF5-7153BE7C205D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="99">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -398,6 +398,9 @@
   </si>
   <si>
     <t>Continuing to trouble shoot fodder_enemy_sm</t>
+  </si>
+  <si>
+    <t>Refactoring state machine</t>
   </si>
 </sst>
 </file>
@@ -536,8 +539,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G78" totalsRowShown="0">
-  <autoFilter ref="B6:G78" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G79" totalsRowShown="0">
+  <autoFilter ref="B6:G79" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
@@ -929,8 +932,8 @@
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>SUM(G7:G78)</f>
-        <v>8.59236111111111</v>
+        <f>SUM(G7:G79)</f>
+        <v>8.1909722222222214</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -2310,6 +2313,9 @@
       <c r="C78" s="2">
         <v>0.45833333333333331</v>
       </c>
+      <c r="D78" s="2">
+        <v>0.59861111111111109</v>
+      </c>
       <c r="E78" t="s">
         <v>74</v>
       </c>
@@ -2318,7 +2324,17 @@
       </c>
       <c r="G78" s="2">
         <f>IF(D78&lt;C78, D78+1, D78) - C78</f>
-        <v>0.54166666666666674</v>
+        <v>0.14027777777777778</v>
+      </c>
+    </row>
+    <row r="79" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C79" s="2"/>
+      <c r="F79" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="G79" s="2">
+        <f>IF(D79&lt;C79, D79+1, D79) - C79</f>
+        <v>0</v>
       </c>
     </row>
     <row r="81" spans="6:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
About to implement state config generation
</commit_message>
<xml_diff>
--- a/Documents/Game Development/Godot/Smash Dungeon/SD_WorkLog.xlsx
+++ b/Documents/Game Development/Godot/Smash Dungeon/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B43942-6166-40D9-ACF5-7153BE7C205D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0C66B25-29C2-4977-8A44-9FAD01356CEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="104">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -400,7 +400,24 @@
     <t>Continuing to trouble shoot fodder_enemy_sm</t>
   </si>
   <si>
-    <t>Refactoring state machine</t>
+    <t>Blog post</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t>blogpost</t>
+  </si>
+  <si>
+    <t>Column3</t>
+  </si>
+  <si>
+    <t>Creating Config states for state machine
+allows better inspector</t>
+  </si>
+  <si>
+    <t>Refactoring state machines
+- mixup with state machines and enum enemy system, parameters are spread across different parts of the inspector</t>
   </si>
 </sst>
 </file>
@@ -410,7 +427,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[h]:mm"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -428,6 +445,12 @@
     <font>
       <sz val="16"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -539,9 +562,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G79" totalsRowShown="0">
-  <autoFilter ref="B6:G79" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:I80" totalsRowShown="0">
+  <autoFilter ref="B6:I80" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
     <tableColumn id="3" xr3:uid="{385CF12C-F475-4237-A1B1-BA2B136D502D}" name="Finish"/>
@@ -550,6 +573,8 @@
     <tableColumn id="6" xr3:uid="{6B5828D5-4B73-426F-9AEB-9B2280524C8F}" name="Time" dataDxfId="6">
       <calculatedColumnFormula>IF(D7&lt;C7, D7+1, D7) - C7</calculatedColumnFormula>
     </tableColumn>
+    <tableColumn id="7" xr3:uid="{5CA719F1-B591-4990-9610-6CFCA1E1664C}" name="Column1"/>
+    <tableColumn id="9" xr3:uid="{0376A738-C71D-4C5D-BB07-AEAE10033BBB}" name="Column3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight18" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -906,7 +931,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I97"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -932,13 +957,9 @@
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>SUM(G7:G79)</f>
-        <v>8.1909722222222214</v>
-      </c>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I5" s="2"/>
+        <f>SUM(G7:G80)</f>
+        <v>8.5243055555555554</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
@@ -959,7 +980,12 @@
       <c r="G6" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="2"/>
+      <c r="H6" t="s">
+        <v>99</v>
+      </c>
+      <c r="I6" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B7" s="1">
@@ -981,7 +1007,6 @@
         <f t="shared" ref="G7:G11" si="0">IF(D7&lt;C7, D7+1, D7) - C7</f>
         <v>0.14930555555555558</v>
       </c>
-      <c r="I7" s="2"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C8" s="2">
@@ -994,7 +1019,6 @@
         <f t="shared" si="0"/>
         <v>0.17152777777777783</v>
       </c>
-      <c r="I8" s="2"/>
     </row>
     <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B9" s="1">
@@ -1016,7 +1040,6 @@
         <f t="shared" si="0"/>
         <v>6.25E-2</v>
       </c>
-      <c r="I9" s="2"/>
     </row>
     <row r="10" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="C10" s="2">
@@ -1035,7 +1058,6 @@
         <f t="shared" si="0"/>
         <v>9.3055555555555558E-2</v>
       </c>
-      <c r="I10" s="2"/>
     </row>
     <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="C11" s="2">
@@ -1154,7 +1176,7 @@
         <v>0.10416666666666663</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" s="1">
         <v>45744</v>
       </c>
@@ -1175,7 +1197,7 @@
         <v>0.25000000000000011</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B18" s="1">
         <v>45745</v>
       </c>
@@ -1196,7 +1218,7 @@
         <v>6.2500000000000056E-2</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:9" ht="60" x14ac:dyDescent="0.25">
       <c r="B19" s="1"/>
       <c r="C19" s="2">
         <v>0.625</v>
@@ -1215,7 +1237,7 @@
         <v>0.16666666666666663</v>
       </c>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="1"/>
       <c r="C20" s="2">
         <v>0.875</v>
@@ -1231,7 +1253,7 @@
         <v>0.5625</v>
       </c>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C21" s="2">
         <v>0.98958333333333337</v>
       </c>
@@ -1246,7 +1268,7 @@
         <v>5.208333333333337E-2</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:9" ht="75" x14ac:dyDescent="0.25">
       <c r="B22" s="1">
         <v>45746</v>
       </c>
@@ -1267,7 +1289,7 @@
         <v>0.11388888888888893</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:9" ht="30" x14ac:dyDescent="0.25">
       <c r="C23" s="2">
         <v>0.79166666666666663</v>
       </c>
@@ -1282,7 +1304,7 @@
         <v>6.597222222222221E-2</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:9" ht="75" x14ac:dyDescent="0.25">
       <c r="B24" s="1">
         <v>45747</v>
       </c>
@@ -1302,8 +1324,11 @@
         <f t="shared" si="2"/>
         <v>9.375E-2</v>
       </c>
-    </row>
-    <row r="25" spans="2:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="I24" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" ht="60" x14ac:dyDescent="0.25">
       <c r="C25" s="2">
         <v>0.75902777777777775</v>
       </c>
@@ -1321,7 +1346,7 @@
         <v>3.125E-2</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:9" ht="45" x14ac:dyDescent="0.25">
       <c r="C26" s="2">
         <v>0.89583333333333337</v>
       </c>
@@ -1339,7 +1364,7 @@
         <v>8.6805555555555469E-2</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:9" ht="45" x14ac:dyDescent="0.25">
       <c r="C27" s="2">
         <v>3.472222222222222E-3</v>
       </c>
@@ -1357,7 +1382,7 @@
         <v>3.125E-2</v>
       </c>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B28" s="1">
         <v>45749</v>
       </c>
@@ -1378,7 +1403,7 @@
         <v>3.472222222222221E-2</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="120" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:9" ht="120" x14ac:dyDescent="0.25">
       <c r="B29" s="1">
         <v>45750</v>
       </c>
@@ -1399,7 +1424,7 @@
         <v>7.5694444444444509E-2</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B30" s="1">
         <v>45751</v>
       </c>
@@ -1420,7 +1445,7 @@
         <v>3.819444444444442E-2</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:9" ht="75" x14ac:dyDescent="0.25">
       <c r="C31" s="2">
         <v>0.88124999999999998</v>
       </c>
@@ -1438,7 +1463,7 @@
         <v>3.0555555555555558E-2</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B32" s="1">
         <v>45752</v>
       </c>
@@ -1459,7 +1484,7 @@
         <v>0.19791666666666663</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:9" ht="45" x14ac:dyDescent="0.25">
       <c r="B33" s="1">
         <v>45753</v>
       </c>
@@ -1480,7 +1505,7 @@
         <v>3.7499999999999978E-2</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:9" ht="60" x14ac:dyDescent="0.25">
       <c r="C34" s="2">
         <v>0.89722222222222225</v>
       </c>
@@ -1498,7 +1523,7 @@
         <v>6.1111111111111116E-2</v>
       </c>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B35" s="1">
         <v>45754</v>
       </c>
@@ -1519,7 +1544,7 @@
         <v>7.2916666666666741E-2</v>
       </c>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B36" s="1"/>
       <c r="C36" s="2">
         <v>0.70833333333333337</v>
@@ -1537,8 +1562,11 @@
         <f t="shared" si="4"/>
         <v>0.16666666666666663</v>
       </c>
-    </row>
-    <row r="37" spans="2:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="I36" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" ht="75" x14ac:dyDescent="0.25">
       <c r="C37" s="2">
         <v>0.89097222222222228</v>
       </c>
@@ -1556,7 +1584,7 @@
         <v>3.9583333333333304E-2</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:9" ht="30" x14ac:dyDescent="0.25">
       <c r="C38" s="2">
         <v>0.98611111111111116</v>
       </c>
@@ -1574,7 +1602,7 @@
         <v>2.0833333333333259E-2</v>
       </c>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B39" s="1">
         <v>45755</v>
       </c>
@@ -1595,7 +1623,7 @@
         <v>5.2777777777777701E-2</v>
       </c>
     </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B40" s="1"/>
       <c r="C40" s="2">
         <v>0.90277777777777779</v>
@@ -1614,7 +1642,7 @@
         <v>4.166666666666663E-2</v>
       </c>
     </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B41" s="1">
         <v>45756</v>
       </c>
@@ -1634,8 +1662,11 @@
         <f>IF(D41&lt;C41, D41+1, D41) - C41</f>
         <v>9.027777777777779E-2</v>
       </c>
-    </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="I41" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
       <c r="C42" s="2">
         <v>0.84513888888888888</v>
@@ -1654,7 +1685,7 @@
         <v>9.2361111111111116E-2</v>
       </c>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B43" s="1">
         <v>45757</v>
       </c>
@@ -1673,7 +1704,7 @@
         <v>0.31944444444444442</v>
       </c>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B44" s="1">
         <v>45758</v>
       </c>
@@ -1694,7 +1725,7 @@
         <v>0.15972222222222221</v>
       </c>
     </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C45" s="2">
         <v>0.66666666666666663</v>
       </c>
@@ -1712,7 +1743,7 @@
         <v>4.1666666666666741E-2</v>
       </c>
     </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C46" s="2">
         <v>0.70833333333333337</v>
       </c>
@@ -1730,7 +1761,7 @@
         <v>4.166666666666663E-2</v>
       </c>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C47" s="2">
         <v>0.75</v>
       </c>
@@ -1748,7 +1779,7 @@
         <v>6.25E-2</v>
       </c>
     </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C48" s="2">
         <v>0.96875</v>
       </c>
@@ -2058,7 +2089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:8" ht="30" x14ac:dyDescent="0.25">
       <c r="B65" s="1">
         <v>45766</v>
       </c>
@@ -2079,7 +2110,7 @@
         <v>0.15972222222222221</v>
       </c>
     </row>
-    <row r="66" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B66" s="1"/>
       <c r="C66" s="2">
         <v>0.66666666666666663</v>
@@ -2098,7 +2129,7 @@
         <v>0.13819444444444451</v>
       </c>
     </row>
-    <row r="67" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B67" s="1"/>
       <c r="C67" s="2">
         <v>0.86805555555555558</v>
@@ -2114,7 +2145,7 @@
         <v>4.8611111111111049E-2</v>
       </c>
     </row>
-    <row r="68" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B68" s="1"/>
       <c r="C68" s="2">
         <v>0.91666666666666663</v>
@@ -2133,7 +2164,7 @@
         <v>9.027777777777779E-2</v>
       </c>
     </row>
-    <row r="69" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B69" s="1">
         <v>45767</v>
       </c>
@@ -2154,7 +2185,7 @@
         <v>8.5416666666666696E-2</v>
       </c>
     </row>
-    <row r="70" spans="2:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:8" ht="60" x14ac:dyDescent="0.25">
       <c r="B70" s="1"/>
       <c r="C70" s="2">
         <v>0.89652777777777781</v>
@@ -2173,7 +2204,7 @@
         <v>0.22777777777777763</v>
       </c>
     </row>
-    <row r="71" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B71" s="1">
         <v>45768</v>
       </c>
@@ -2192,7 +2223,7 @@
         <v>0.59027777777777779</v>
       </c>
     </row>
-    <row r="72" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B72" s="1"/>
       <c r="C72" s="2"/>
       <c r="D72" s="2"/>
@@ -2207,7 +2238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B73" s="1">
         <v>45769</v>
       </c>
@@ -2228,7 +2259,7 @@
         <v>0.28749999999999998</v>
       </c>
     </row>
-    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C74" s="2">
         <v>0.97916666666666663</v>
       </c>
@@ -2246,7 +2277,7 @@
         <v>8.9583333333333459E-2</v>
       </c>
     </row>
-    <row r="75" spans="2:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:8" ht="45" x14ac:dyDescent="0.25">
       <c r="B75" s="1">
         <v>45770</v>
       </c>
@@ -2267,7 +2298,7 @@
         <v>0.18055555555555558</v>
       </c>
     </row>
-    <row r="76" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:8" ht="30" x14ac:dyDescent="0.25">
       <c r="C76" s="2">
         <v>0.9375</v>
       </c>
@@ -2285,7 +2316,7 @@
         <v>4.166666666666663E-2</v>
       </c>
     </row>
-    <row r="77" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B77" s="1">
         <v>45772</v>
       </c>
@@ -2306,7 +2337,7 @@
         <v>0.10000000000000009</v>
       </c>
     </row>
-    <row r="78" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B78" s="1">
         <v>45773</v>
       </c>
@@ -2327,27 +2358,107 @@
         <v>0.14027777777777778</v>
       </c>
     </row>
-    <row r="79" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C79" s="2"/>
+    <row r="79" spans="2:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="C79" s="2">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="D79" s="2">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="E79" t="s">
+        <v>74</v>
+      </c>
       <c r="F79" s="3" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="G79" s="2">
         <f>IF(D79&lt;C79, D79+1, D79) - C79</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F81" s="8" t="s">
+        <v>0.125</v>
+      </c>
+      <c r="H79" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="80" spans="2:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="C80" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F80" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G80" s="2">
+        <f>IF(D80&lt;C80, D80+1, D80) - C80</f>
+        <v>0.20833333333333337</v>
+      </c>
+    </row>
+    <row r="81" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C81" s="2"/>
+      <c r="G81" s="2"/>
+    </row>
+    <row r="82" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C82" s="2"/>
+      <c r="G82" s="2"/>
+    </row>
+    <row r="83" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C83" s="2"/>
+      <c r="G83" s="2"/>
+    </row>
+    <row r="84" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C84" s="2"/>
+      <c r="G84" s="2"/>
+    </row>
+    <row r="85" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C85" s="2"/>
+      <c r="G85" s="2"/>
+    </row>
+    <row r="86" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C86" s="2"/>
+      <c r="G86" s="2"/>
+    </row>
+    <row r="87" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C87" s="2"/>
+      <c r="G87" s="2"/>
+    </row>
+    <row r="88" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C88" s="2"/>
+      <c r="G88" s="2"/>
+    </row>
+    <row r="89" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C89" s="2"/>
+      <c r="G89" s="2"/>
+    </row>
+    <row r="90" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C90" s="2"/>
+      <c r="G90" s="2"/>
+    </row>
+    <row r="91" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C91" s="2"/>
+      <c r="G91" s="2"/>
+    </row>
+    <row r="92" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C92" s="2"/>
+      <c r="G92" s="2"/>
+    </row>
+    <row r="93" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C93" s="2"/>
+      <c r="G93" s="2"/>
+    </row>
+    <row r="94" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C94" s="2"/>
+      <c r="G94" s="2"/>
+    </row>
+    <row r="96" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="F96" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="82" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F82" s="9" t="s">
+    <row r="97" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F97" s="9" t="s">
         <v>42</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">

</xml_diff>